<commit_message>
22127410: test case updated
</commit_message>
<xml_diff>
--- a/project/HW3/22127410/22127410_DataGeneration_10/22127410_BugReport.xlsx
+++ b/project/HW3/22127410/22127410_DataGeneration_10/22127410_BugReport.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/thanhthuy/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/thanhthuy/Documents/Testing-PRJ-SM/project/HW3/22127410/22127410_DataGeneration_10/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A79135E-245A-7E45-B477-EBE26B184397}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8BCA5CF-3093-E34C-A95F-02D1D53EB144}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="18380" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="18360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Test summary report" sheetId="1" r:id="rId1"/>
@@ -749,7 +749,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -773,32 +773,11 @@
     <xf numFmtId="14" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="16">
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-      </font>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
     <dxf>
       <font>
         <strike val="0"/>
@@ -876,6 +855,18 @@
         <name val="Arial"/>
         <family val="2"/>
         <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
       </font>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -1136,22 +1127,22 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table3" displayName="Table3" ref="A1:N20" totalsRowShown="0" headerRowDxfId="15" dataDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table3" displayName="Table3" ref="A1:N20" totalsRowShown="0" headerRowDxfId="15" dataDxfId="14">
   <tableColumns count="14">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Defect ID" dataDxfId="14"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Defect Title" dataDxfId="13"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Defect Description" dataDxfId="12"/>
-    <tableColumn id="2" xr3:uid="{481DB5E1-8C0A-1141-BE4B-253435B69B8C}" name="Steps to Reproduce" dataDxfId="11"/>
-    <tableColumn id="4" xr3:uid="{29F06308-5E19-B442-BFD9-F2A1F77FCD64}" name="Expected Result" dataDxfId="10"/>
-    <tableColumn id="7" xr3:uid="{ACDC4036-2AFE-8741-B938-4C882D635CA7}" name="Actual Result" dataDxfId="9"/>
-    <tableColumn id="14" xr3:uid="{538B3C11-634B-9443-BF24-DD5F74863919}" name="Screenshots" dataDxfId="8"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Feature ID" dataDxfId="7"/>
-    <tableColumn id="13" xr3:uid="{7F7C74B9-E67B-C741-BC60-B0D22D903146}" name="Severity" dataDxfId="6"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Priority" dataDxfId="5"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Reported By" dataDxfId="4"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Date Reported" dataDxfId="3"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Status" dataDxfId="2"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Comment" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Defect ID" dataDxfId="13"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Defect Title" dataDxfId="12"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Defect Description" dataDxfId="11"/>
+    <tableColumn id="2" xr3:uid="{481DB5E1-8C0A-1141-BE4B-253435B69B8C}" name="Steps to Reproduce" dataDxfId="10"/>
+    <tableColumn id="4" xr3:uid="{29F06308-5E19-B442-BFD9-F2A1F77FCD64}" name="Expected Result" dataDxfId="9"/>
+    <tableColumn id="7" xr3:uid="{ACDC4036-2AFE-8741-B938-4C882D635CA7}" name="Actual Result" dataDxfId="8"/>
+    <tableColumn id="14" xr3:uid="{538B3C11-634B-9443-BF24-DD5F74863919}" name="Screenshots" dataDxfId="7"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Feature ID" dataDxfId="6"/>
+    <tableColumn id="13" xr3:uid="{7F7C74B9-E67B-C741-BC60-B0D22D903146}" name="Severity" dataDxfId="5"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Priority" dataDxfId="4"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Reported By" dataDxfId="3"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Date Reported" dataDxfId="2"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Status" dataDxfId="1"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Comment" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1465,7 +1456,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="8">
-        <v>45831</v>
+        <v>45830</v>
       </c>
       <c r="C2" s="8"/>
       <c r="D2" s="8"/>
@@ -2163,7 +2154,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="1:14" ht="97" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:13" ht="97" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="4" t="s">
         <v>32</v>
       </c>
@@ -2204,7 +2195,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="18" spans="1:14" ht="98" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:13" ht="98" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="4"/>
       <c r="B18" s="1" t="s">
         <v>107</v>
@@ -2243,7 +2234,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="19" spans="1:14" ht="97" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:13" ht="97" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="4"/>
       <c r="B19" s="1" t="s">
         <v>112</v>
@@ -2282,8 +2273,8 @@
         <v>12</v>
       </c>
     </row>
-    <row r="20" spans="1:14" ht="97" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="9"/>
+    <row r="20" spans="1:13" ht="97" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="4"/>
       <c r="B20" s="1" t="s">
         <v>116</v>
       </c>
@@ -2320,20 +2311,16 @@
       <c r="M20" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N20" s="10"/>
-    </row>
-    <row r="21" spans="1:14" ht="97" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="9"/>
+    </row>
+    <row r="21" spans="1:13" ht="97" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="4"/>
       <c r="G21"/>
       <c r="H21"/>
       <c r="I21"/>
       <c r="J21"/>
-      <c r="K21" s="10"/>
-      <c r="L21" s="11"/>
-      <c r="M21" s="10"/>
-      <c r="N21" s="10"/>
-    </row>
-    <row r="22" spans="1:14" ht="96" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L21" s="3"/>
+    </row>
+    <row r="22" spans="1:13" ht="96" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="4"/>
       <c r="B22" s="5"/>
       <c r="C22" s="5"/>
@@ -2345,7 +2332,7 @@
       <c r="J22" s="5"/>
       <c r="L22" s="6"/>
     </row>
-    <row r="23" spans="1:14" ht="98" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:13" ht="98" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="4"/>
       <c r="B23" s="5"/>
       <c r="C23" s="5"/>
@@ -2357,7 +2344,7 @@
       <c r="J23" s="5"/>
       <c r="L23" s="6"/>
     </row>
-    <row r="24" spans="1:14" ht="99" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:13" ht="99" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="4"/>
       <c r="B24" s="5"/>
       <c r="C24" s="5"/>
@@ -2369,7 +2356,7 @@
       <c r="J24" s="5"/>
       <c r="L24" s="6"/>
     </row>
-    <row r="25" spans="1:14" ht="97" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:13" ht="97" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="4"/>
       <c r="B25" s="5"/>
       <c r="C25" s="5"/>
@@ -2381,7 +2368,7 @@
       <c r="J25" s="5"/>
       <c r="L25" s="6"/>
     </row>
-    <row r="26" spans="1:14" ht="98" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:13" ht="98" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="4"/>
       <c r="B26" s="5"/>
       <c r="C26" s="5"/>
@@ -2393,7 +2380,7 @@
       <c r="J26" s="5"/>
       <c r="L26" s="6"/>
     </row>
-    <row r="27" spans="1:14" ht="98" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:13" ht="98" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="4"/>
       <c r="B27" s="5"/>
       <c r="C27" s="5"/>
@@ -2405,7 +2392,7 @@
       <c r="J27" s="5"/>
       <c r="L27" s="6"/>
     </row>
-    <row r="28" spans="1:14" ht="98" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:13" ht="98" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="4"/>
       <c r="B28" s="5"/>
       <c r="C28" s="5"/>
@@ -2417,7 +2404,7 @@
       <c r="J28" s="5"/>
       <c r="L28" s="6"/>
     </row>
-    <row r="29" spans="1:14" ht="97" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:13" ht="97" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="4"/>
       <c r="B29" s="5"/>
       <c r="C29" s="5"/>
@@ -2429,7 +2416,7 @@
       <c r="J29" s="5"/>
       <c r="L29" s="6"/>
     </row>
-    <row r="30" spans="1:14" ht="97" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:13" ht="97" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="4"/>
       <c r="B30" s="5"/>
       <c r="C30" s="5"/>
@@ -2441,7 +2428,7 @@
       <c r="J30" s="5"/>
       <c r="L30" s="6"/>
     </row>
-    <row r="31" spans="1:14" ht="100" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:13" ht="100" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="4"/>
       <c r="B31" s="5"/>
       <c r="C31" s="5"/>
@@ -2453,7 +2440,7 @@
       <c r="J31" s="5"/>
       <c r="L31" s="6"/>
     </row>
-    <row r="32" spans="1:14" ht="99" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:13" ht="99" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="4"/>
       <c r="B32" s="5"/>
       <c r="C32" s="5"/>

</xml_diff>